<commit_message>
audit(2026-06-08): update PRs sheet with PR #164
</commit_message>
<xml_diff>
--- a/audits/daily_usability_audit_2026-06-08.xlsx
+++ b/audits/daily_usability_audit_2026-06-08.xlsx
@@ -97,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,6 +115,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -10826,14 +10829,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="95" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10860,6 +10863,87 @@
       <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Issues fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>funder-finder</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>164</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>usability/2026-06-08-fixes</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>https://github.com/SpikeyCoder/funder-finder/pull/164</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>Audit report only — no standard 8-category usability bugs found this cycle. All Instrumentl gap FAILs/PARTIALs are deferred to fundermatch-feature-builder per scheduled-task spec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>my_website</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>(no PR)</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>No usability bugs found in standard 8-category audit. KAR-A11Y-012 subheader green is owner-approved exception. KAR-NAV-010 amazon.co.uk returned 429 (rate limit, not 404).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>chaos_tester</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>(no PR)</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>No usability bugs found in standard 8-category audit. WAO-NAV-011 /healthz returning 404 on live is a deploy lag (route defined in app.py L950); /api/health works correctly.</t>
         </is>
       </c>
     </row>

</xml_diff>